<commit_message>
Actualizar reporte - Comparativo (vs ventas)
</commit_message>
<xml_diff>
--- a/shared_uploads/vsventas.xlsx
+++ b/shared_uploads/vsventas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\C960806\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4EF19B9-2793-4DA3-9924-3EBE88E6EE15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA705CFD-5D7A-4DD6-8449-C116939289A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9727" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10015" uniqueCount="117">
   <si>
     <t># Mes</t>
   </si>
@@ -80130,7 +80130,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE92DB44-9108-48C0-9E4D-CDD7D4A1EECC}">
-  <dimension ref="A1:K379"/>
+  <dimension ref="A1:K475"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.90625" style="5"/>
@@ -88988,22 +88988,22 @@
         <v>10</v>
       </c>
       <c r="F291" s="2">
-        <v>56814105.280000001</v>
+        <v>118726877.58</v>
       </c>
       <c r="G291" s="2">
-        <v>838783.9</v>
+        <v>1521118.2</v>
       </c>
       <c r="H291" s="2">
-        <v>44412514.939999998</v>
+        <v>92685126.030000001</v>
       </c>
       <c r="I291" s="2">
-        <v>636325.31000000006</v>
+        <v>1168629.3799999999</v>
       </c>
       <c r="J291" s="3">
-        <v>114</v>
+        <v>349</v>
       </c>
       <c r="K291" s="3">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="292" spans="1:11" x14ac:dyDescent="0.25">
@@ -89023,11 +89023,11 @@
         <v>11</v>
       </c>
       <c r="F292" s="2">
-        <v>51309425.82</v>
+        <v>111150122.16</v>
       </c>
       <c r="G292"/>
       <c r="H292" s="2">
-        <v>40167811.240000002</v>
+        <v>86923231.939999998</v>
       </c>
       <c r="I292"/>
     </row>
@@ -89048,22 +89048,22 @@
         <v>12</v>
       </c>
       <c r="F293" s="2">
-        <v>53587224.149999999</v>
+        <v>94763689.629999995</v>
       </c>
       <c r="G293" s="2">
-        <v>1169657.06</v>
+        <v>629660.06000000006</v>
       </c>
       <c r="H293" s="2">
-        <v>42277267.229999997</v>
+        <v>74609062.469999999</v>
       </c>
       <c r="I293" s="2">
-        <v>918904.47</v>
+        <v>500518.35</v>
       </c>
       <c r="J293" s="3">
-        <v>305.53199999999998</v>
+        <v>301.53199999999998</v>
       </c>
       <c r="K293" s="3">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="294" spans="1:11" x14ac:dyDescent="0.25">
@@ -89083,11 +89083,11 @@
         <v>13</v>
       </c>
       <c r="F294" s="2">
-        <v>44794424.859999999</v>
+        <v>83541223.540000007</v>
       </c>
       <c r="G294"/>
       <c r="H294" s="2">
-        <v>35352710.649999999</v>
+        <v>65612183.329999998</v>
       </c>
       <c r="I294"/>
     </row>
@@ -89108,11 +89108,11 @@
         <v>14</v>
       </c>
       <c r="F295" s="2">
-        <v>48738620.170000002</v>
+        <v>93414161.099999994</v>
       </c>
       <c r="G295"/>
       <c r="H295" s="2">
-        <v>38150513.380000003</v>
+        <v>73065540.049999997</v>
       </c>
       <c r="I295"/>
     </row>
@@ -89133,11 +89133,11 @@
         <v>16</v>
       </c>
       <c r="F296" s="2">
-        <v>69158414.689999998</v>
+        <v>138201218.75</v>
       </c>
       <c r="G296"/>
       <c r="H296" s="2">
-        <v>54343172.049999997</v>
+        <v>108273701.16</v>
       </c>
       <c r="I296"/>
     </row>
@@ -89158,11 +89158,11 @@
         <v>17</v>
       </c>
       <c r="F297" s="2">
-        <v>34705327.340000004</v>
+        <v>57417149.240000002</v>
       </c>
       <c r="G297"/>
       <c r="H297" s="2">
-        <v>27212043.440000001</v>
+        <v>45045172.229999997</v>
       </c>
       <c r="I297"/>
     </row>
@@ -89183,11 +89183,11 @@
         <v>18</v>
       </c>
       <c r="F298" s="2">
-        <v>45716472.630000003</v>
+        <v>73691626.819999993</v>
       </c>
       <c r="G298"/>
       <c r="H298" s="2">
-        <v>36555814.740000002</v>
+        <v>58555557.990000002</v>
       </c>
       <c r="I298"/>
     </row>
@@ -89208,11 +89208,11 @@
         <v>19</v>
       </c>
       <c r="F299" s="2">
-        <v>35131909.030000001</v>
+        <v>73364071.069999993</v>
       </c>
       <c r="G299"/>
       <c r="H299" s="2">
-        <v>27533147.629999999</v>
+        <v>57407689.549999997</v>
       </c>
       <c r="I299"/>
     </row>
@@ -89233,11 +89233,11 @@
         <v>20</v>
       </c>
       <c r="F300" s="2">
-        <v>42923910.039999999</v>
+        <v>72802202.319999993</v>
       </c>
       <c r="G300"/>
       <c r="H300" s="2">
-        <v>33838330.719999999</v>
+        <v>57331206.090000004</v>
       </c>
       <c r="I300"/>
     </row>
@@ -89258,11 +89258,11 @@
         <v>21</v>
       </c>
       <c r="F301" s="2">
-        <v>37800498.270000003</v>
+        <v>72259010.530000001</v>
       </c>
       <c r="G301"/>
       <c r="H301" s="2">
-        <v>29650561.350000001</v>
+        <v>56595522.509999998</v>
       </c>
       <c r="I301"/>
     </row>
@@ -89283,11 +89283,11 @@
         <v>22</v>
       </c>
       <c r="F302" s="2">
-        <v>35087569.219999999</v>
+        <v>68405062.510000005</v>
       </c>
       <c r="G302"/>
       <c r="H302" s="2">
-        <v>27570687.260000002</v>
+        <v>53778765.969999999</v>
       </c>
       <c r="I302"/>
     </row>
@@ -89308,11 +89308,11 @@
         <v>23</v>
       </c>
       <c r="F303" s="2">
-        <v>61908259.509999998</v>
+        <v>118779902.66</v>
       </c>
       <c r="G303"/>
       <c r="H303" s="2">
-        <v>48501538.939999998</v>
+        <v>92946858.579999998</v>
       </c>
       <c r="I303"/>
     </row>
@@ -89333,13 +89333,13 @@
         <v>24</v>
       </c>
       <c r="F304" s="2">
-        <v>57380799.770000003</v>
+        <v>101771190.23</v>
       </c>
       <c r="G304" s="2">
         <v>699999</v>
       </c>
       <c r="H304" s="2">
-        <v>44827338.140000001</v>
+        <v>79652500.260000005</v>
       </c>
       <c r="I304" s="2">
         <v>542354.63</v>
@@ -89368,13 +89368,13 @@
         <v>25</v>
       </c>
       <c r="F305" s="2">
-        <v>29992610.789999999</v>
+        <v>48471306.420000002</v>
       </c>
       <c r="G305" s="2">
         <v>104105.05</v>
       </c>
       <c r="H305" s="2">
-        <v>23574669.57</v>
+        <v>38072373.130000003</v>
       </c>
       <c r="I305" s="2">
         <v>80887.320000000007</v>
@@ -89403,11 +89403,11 @@
         <v>26</v>
       </c>
       <c r="F306" s="2">
-        <v>41685684.840000004</v>
+        <v>79583941.840000004</v>
       </c>
       <c r="G306"/>
       <c r="H306" s="2">
-        <v>32874598.09</v>
+        <v>62456281.920000002</v>
       </c>
       <c r="I306"/>
     </row>
@@ -89428,11 +89428,11 @@
         <v>27</v>
       </c>
       <c r="F307" s="2">
-        <v>33124046.25</v>
+        <v>64513349.060000002</v>
       </c>
       <c r="G307"/>
       <c r="H307" s="2">
-        <v>26085163.050000001</v>
+        <v>50489975.939999998</v>
       </c>
       <c r="I307"/>
     </row>
@@ -89453,13 +89453,13 @@
         <v>28</v>
       </c>
       <c r="F308" s="2">
-        <v>65247870.490000002</v>
+        <v>117796011.15000001</v>
       </c>
       <c r="G308" s="2">
         <v>91668.5</v>
       </c>
       <c r="H308" s="2">
-        <v>51623501.490000002</v>
+        <v>93167711.340000004</v>
       </c>
       <c r="I308" s="2">
         <v>77773.06</v>
@@ -89488,13 +89488,13 @@
         <v>30</v>
       </c>
       <c r="F309" s="2">
-        <v>64622392.539999999</v>
+        <v>117266827.05</v>
       </c>
       <c r="G309" s="2">
         <v>559301.42000000004</v>
       </c>
       <c r="H309" s="2">
-        <v>50636690.57</v>
+        <v>91732089.5</v>
       </c>
       <c r="I309" s="2">
         <v>433825.97</v>
@@ -89523,11 +89523,11 @@
         <v>31</v>
       </c>
       <c r="F310" s="2">
-        <v>41591563.649999999</v>
+        <v>76798351.090000004</v>
       </c>
       <c r="G310"/>
       <c r="H310" s="2">
-        <v>32859983.609999999</v>
+        <v>60462892</v>
       </c>
       <c r="I310"/>
     </row>
@@ -89548,11 +89548,11 @@
         <v>32</v>
       </c>
       <c r="F311" s="2">
-        <v>12369537.91</v>
+        <v>19439096.559999999</v>
       </c>
       <c r="G311"/>
       <c r="H311" s="2">
-        <v>9823496</v>
+        <v>15396886.949999999</v>
       </c>
       <c r="I311"/>
     </row>
@@ -89573,11 +89573,11 @@
         <v>33</v>
       </c>
       <c r="F312" s="2">
-        <v>35378530.020000003</v>
+        <v>55949713.020000003</v>
       </c>
       <c r="G312"/>
       <c r="H312" s="2">
-        <v>27862050.66</v>
+        <v>44014945.5</v>
       </c>
       <c r="I312"/>
     </row>
@@ -89598,11 +89598,11 @@
         <v>34</v>
       </c>
       <c r="F313" s="2">
-        <v>30459227.34</v>
+        <v>56223519.640000001</v>
       </c>
       <c r="G313"/>
       <c r="H313" s="2">
-        <v>24066289.16</v>
+        <v>44303238.240000002</v>
       </c>
       <c r="I313"/>
     </row>
@@ -89623,11 +89623,11 @@
         <v>35</v>
       </c>
       <c r="F314" s="2">
-        <v>14788412.9</v>
+        <v>24928004.879999999</v>
       </c>
       <c r="G314"/>
       <c r="H314" s="2">
-        <v>11752156.380000001</v>
+        <v>19778846.420000002</v>
       </c>
       <c r="I314"/>
     </row>
@@ -89648,11 +89648,11 @@
         <v>36</v>
       </c>
       <c r="F315" s="2">
-        <v>60911503.920000002</v>
+        <v>61364373.060000002</v>
       </c>
       <c r="G315"/>
       <c r="H315" s="2">
-        <v>48608347.170000002</v>
+        <v>48971795.340000004</v>
       </c>
       <c r="I315"/>
     </row>
@@ -89673,11 +89673,11 @@
         <v>37</v>
       </c>
       <c r="F316" s="2">
-        <v>42173516.729999997</v>
+        <v>70906267.519999996</v>
       </c>
       <c r="G316"/>
       <c r="H316" s="2">
-        <v>33203102.640000001</v>
+        <v>55715973.399999999</v>
       </c>
       <c r="I316"/>
     </row>
@@ -89698,22 +89698,22 @@
         <v>38</v>
       </c>
       <c r="F317" s="2">
-        <v>37427368.789999999</v>
+        <v>64174373.590000004</v>
       </c>
       <c r="G317" s="2">
-        <v>1064539.1499999999</v>
+        <v>2014409.35</v>
       </c>
       <c r="H317" s="2">
-        <v>29545466.859999999</v>
+        <v>50586661.299999997</v>
       </c>
       <c r="I317" s="2">
-        <v>827490.12</v>
+        <v>1563443.33</v>
       </c>
       <c r="J317" s="3">
-        <v>24</v>
+        <v>43</v>
       </c>
       <c r="K317" s="3">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="318" spans="1:11" x14ac:dyDescent="0.25">
@@ -89733,13 +89733,13 @@
         <v>39</v>
       </c>
       <c r="F318" s="2">
-        <v>25514009.050000001</v>
+        <v>45669484.539999999</v>
       </c>
       <c r="G318" s="2">
         <v>-91413.75</v>
       </c>
       <c r="H318" s="2">
-        <v>20067749.219999999</v>
+        <v>35903073.640000001</v>
       </c>
       <c r="I318" s="2">
         <v>-76951.820000000007</v>
@@ -89768,11 +89768,11 @@
         <v>40</v>
       </c>
       <c r="F319" s="2">
-        <v>7037528.0899999999</v>
+        <v>7386000.7999999998</v>
       </c>
       <c r="G319"/>
       <c r="H319" s="2">
-        <v>5541309</v>
+        <v>5819696.8099999996</v>
       </c>
       <c r="I319"/>
     </row>
@@ -89793,13 +89793,13 @@
         <v>43</v>
       </c>
       <c r="F320" s="2">
-        <v>45248968.32</v>
+        <v>89089111.549999997</v>
       </c>
       <c r="G320" s="2">
         <v>2349998.19</v>
       </c>
       <c r="H320" s="2">
-        <v>35353148.369999997</v>
+        <v>69402407.099999994</v>
       </c>
       <c r="I320" s="2">
         <v>1820763.07</v>
@@ -89828,13 +89828,13 @@
         <v>44</v>
       </c>
       <c r="F321" s="2">
-        <v>35231703.619999997</v>
+        <v>67603087.439999998</v>
       </c>
       <c r="G321" s="2">
         <v>350483.85</v>
       </c>
       <c r="H321" s="2">
-        <v>27873864.949999999</v>
+        <v>53269959.079999998</v>
       </c>
       <c r="I321" s="2">
         <v>272899.42</v>
@@ -89863,11 +89863,11 @@
         <v>45</v>
       </c>
       <c r="F322" s="2">
-        <v>35830746</v>
+        <v>68039540.900000006</v>
       </c>
       <c r="G322"/>
       <c r="H322" s="2">
-        <v>28124638.07</v>
+        <v>53389375.109999999</v>
       </c>
       <c r="I322"/>
     </row>
@@ -89888,11 +89888,11 @@
         <v>46</v>
       </c>
       <c r="F323" s="2">
-        <v>11122852.09</v>
+        <v>19329765.57</v>
       </c>
       <c r="G323"/>
       <c r="H323" s="2">
-        <v>8747218.1799999997</v>
+        <v>15193316.33</v>
       </c>
       <c r="I323"/>
     </row>
@@ -89913,11 +89913,11 @@
         <v>47</v>
       </c>
       <c r="F324" s="2">
-        <v>10040423.449999999</v>
+        <v>15181122.609999999</v>
       </c>
       <c r="G324"/>
       <c r="H324" s="2">
-        <v>7943015.4100000001</v>
+        <v>11987023.869999999</v>
       </c>
       <c r="I324"/>
     </row>
@@ -89938,13 +89938,13 @@
         <v>48</v>
       </c>
       <c r="F325" s="2">
-        <v>11010337.869999999</v>
+        <v>19167614.100000001</v>
       </c>
       <c r="G325" s="2">
         <v>17760</v>
       </c>
       <c r="H325" s="2">
-        <v>8636093.3399999999</v>
+        <v>15036189.43</v>
       </c>
       <c r="I325" s="2">
         <v>13760.32</v>
@@ -89973,11 +89973,11 @@
         <v>49</v>
       </c>
       <c r="F326" s="2">
-        <v>27527320.640000001</v>
+        <v>46560201.509999998</v>
       </c>
       <c r="G326"/>
       <c r="H326" s="2">
-        <v>21481914.579999998</v>
+        <v>36509994.109999999</v>
       </c>
       <c r="I326"/>
     </row>
@@ -89998,13 +89998,23 @@
         <v>50</v>
       </c>
       <c r="F327" s="2">
-        <v>52388130.969999999</v>
-      </c>
-      <c r="G327"/>
+        <v>92895827.349999994</v>
+      </c>
+      <c r="G327">
+        <v>69901.100000000006</v>
+      </c>
       <c r="H327" s="2">
-        <v>41749547.799999997</v>
-      </c>
-      <c r="I327"/>
+        <v>73547274.019999996</v>
+      </c>
+      <c r="I327">
+        <v>54158.94</v>
+      </c>
+      <c r="J327">
+        <v>10</v>
+      </c>
+      <c r="K327">
+        <v>2</v>
+      </c>
     </row>
     <row r="328" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A328" t="s">
@@ -90023,13 +90033,13 @@
         <v>51</v>
       </c>
       <c r="F328" s="2">
-        <v>38850188.340000004</v>
+        <v>64322688.090000004</v>
       </c>
       <c r="G328" s="2">
         <v>80790.5</v>
       </c>
       <c r="H328" s="2">
-        <v>31084626.989999998</v>
+        <v>51032299.420000002</v>
       </c>
       <c r="I328" s="2">
         <v>68543.97</v>
@@ -90058,11 +90068,11 @@
         <v>52</v>
       </c>
       <c r="F329" s="2">
-        <v>31005651.460000001</v>
+        <v>68194640.859999999</v>
       </c>
       <c r="G329"/>
       <c r="H329" s="2">
-        <v>24312870.510000002</v>
+        <v>53512092.549999997</v>
       </c>
       <c r="I329"/>
     </row>
@@ -90083,11 +90093,11 @@
         <v>53</v>
       </c>
       <c r="F330" s="2">
-        <v>32820384.309999999</v>
+        <v>71183622.629999995</v>
       </c>
       <c r="G330"/>
       <c r="H330" s="2">
-        <v>25697133.859999999</v>
+        <v>55677954.649999999</v>
       </c>
       <c r="I330"/>
     </row>
@@ -90108,11 +90118,11 @@
         <v>54</v>
       </c>
       <c r="F331" s="2">
-        <v>28037072.550000001</v>
+        <v>54343883.729999997</v>
       </c>
       <c r="G331"/>
       <c r="H331" s="2">
-        <v>22159882.57</v>
+        <v>42794445.810000002</v>
       </c>
       <c r="I331"/>
     </row>
@@ -90133,11 +90143,11 @@
         <v>55</v>
       </c>
       <c r="F332" s="2">
-        <v>25255417.02</v>
+        <v>47210907.909999996</v>
       </c>
       <c r="G332"/>
       <c r="H332" s="2">
-        <v>19906621.489999998</v>
+        <v>37161048.479999997</v>
       </c>
       <c r="I332"/>
     </row>
@@ -90158,11 +90168,11 @@
         <v>56</v>
       </c>
       <c r="F333" s="2">
-        <v>59028340.719999999</v>
+        <v>124576567.90000001</v>
       </c>
       <c r="G333"/>
       <c r="H333" s="2">
-        <v>46276457.460000001</v>
+        <v>97533818.010000005</v>
       </c>
       <c r="I333"/>
     </row>
@@ -90183,11 +90193,11 @@
         <v>57</v>
       </c>
       <c r="F334" s="2">
-        <v>42515591.869999997</v>
+        <v>74204320.099999994</v>
       </c>
       <c r="G334"/>
       <c r="H334" s="2">
-        <v>33450122.280000001</v>
+        <v>58076161.130000003</v>
       </c>
       <c r="I334"/>
     </row>
@@ -90208,11 +90218,11 @@
         <v>58</v>
       </c>
       <c r="F335" s="2">
-        <v>35393171.619999997</v>
+        <v>62440647.060000002</v>
       </c>
       <c r="G335"/>
       <c r="H335" s="2">
-        <v>27738379.699999999</v>
+        <v>48938952</v>
       </c>
       <c r="I335"/>
     </row>
@@ -90233,11 +90243,11 @@
         <v>59</v>
       </c>
       <c r="F336" s="2">
-        <v>26836684.539999999</v>
+        <v>40216782.479999997</v>
       </c>
       <c r="G336"/>
       <c r="H336" s="2">
-        <v>21387515.27</v>
+        <v>31848878.530000001</v>
       </c>
       <c r="I336"/>
     </row>
@@ -90258,11 +90268,11 @@
         <v>60</v>
       </c>
       <c r="F337" s="2">
-        <v>31680730.289999999</v>
+        <v>69629398.280000001</v>
       </c>
       <c r="G337"/>
       <c r="H337" s="2">
-        <v>24686024.780000001</v>
+        <v>54255233.100000001</v>
       </c>
       <c r="I337"/>
     </row>
@@ -90283,11 +90293,11 @@
         <v>111</v>
       </c>
       <c r="F338" s="2">
-        <v>2188836.2599999998</v>
+        <v>4325526.8099999996</v>
       </c>
       <c r="G338"/>
       <c r="H338" s="2">
-        <v>1706732.36</v>
+        <v>3386241.17</v>
       </c>
       <c r="I338"/>
     </row>
@@ -90308,13 +90318,13 @@
         <v>61</v>
       </c>
       <c r="F339" s="2">
-        <v>26443154.73</v>
+        <v>47184114.289999999</v>
       </c>
       <c r="G339" s="2">
         <v>141823.20000000001</v>
       </c>
       <c r="H339" s="2">
-        <v>20763552</v>
+        <v>36951804.219999999</v>
       </c>
       <c r="I339" s="2">
         <v>109883.52</v>
@@ -90343,11 +90353,11 @@
         <v>62</v>
       </c>
       <c r="F340" s="2">
-        <v>49461759.57</v>
+        <v>85312045.349999994</v>
       </c>
       <c r="G340"/>
       <c r="H340" s="2">
-        <v>38915429.170000002</v>
+        <v>67130046.700000003</v>
       </c>
       <c r="I340"/>
     </row>
@@ -90368,11 +90378,11 @@
         <v>63</v>
       </c>
       <c r="F341" s="2">
-        <v>19877881.280000001</v>
+        <v>31431825.43</v>
       </c>
       <c r="G341"/>
       <c r="H341" s="2">
-        <v>15555791.380000001</v>
+        <v>24590813.43</v>
       </c>
       <c r="I341"/>
     </row>
@@ -90393,11 +90403,11 @@
         <v>64</v>
       </c>
       <c r="F342" s="2">
-        <v>40937563.829999998</v>
+        <v>68761711.209999993</v>
       </c>
       <c r="G342"/>
       <c r="H342" s="2">
-        <v>32592393.859999999</v>
+        <v>54575115.469999999</v>
       </c>
       <c r="I342"/>
     </row>
@@ -90418,11 +90428,11 @@
         <v>65</v>
       </c>
       <c r="F343" s="2">
-        <v>36486712.670000002</v>
+        <v>64137821.170000002</v>
       </c>
       <c r="G343"/>
       <c r="H343" s="2">
-        <v>28766577.93</v>
+        <v>50489816.049999997</v>
       </c>
       <c r="I343"/>
     </row>
@@ -90443,13 +90453,13 @@
         <v>67</v>
       </c>
       <c r="F344" s="2">
-        <v>44401623.740000002</v>
+        <v>75919953.510000005</v>
       </c>
       <c r="G344" s="2">
         <v>129382.78</v>
       </c>
       <c r="H344" s="2">
-        <v>35335077.259999998</v>
+        <v>60049123.460000001</v>
       </c>
       <c r="I344" s="2">
         <v>96370.84</v>
@@ -90478,11 +90488,11 @@
         <v>68</v>
       </c>
       <c r="F345" s="2">
-        <v>37740036.829999998</v>
+        <v>66709045.520000003</v>
       </c>
       <c r="G345"/>
       <c r="H345" s="2">
-        <v>29560958.120000001</v>
+        <v>52155867.079999998</v>
       </c>
       <c r="I345"/>
     </row>
@@ -90503,11 +90513,11 @@
         <v>69</v>
       </c>
       <c r="F346" s="2">
-        <v>26374265.920000002</v>
+        <v>46783420.539999999</v>
       </c>
       <c r="G346"/>
       <c r="H346" s="2">
-        <v>20616714.949999999</v>
+        <v>36606518.450000003</v>
       </c>
       <c r="I346"/>
     </row>
@@ -90528,11 +90538,11 @@
         <v>70</v>
       </c>
       <c r="F347" s="2">
-        <v>16240307.5</v>
+        <v>24744860.949999999</v>
       </c>
       <c r="G347"/>
       <c r="H347" s="2">
-        <v>12906928.85</v>
+        <v>19568588.460000001</v>
       </c>
       <c r="I347"/>
     </row>
@@ -90553,13 +90563,13 @@
         <v>71</v>
       </c>
       <c r="F348" s="2">
-        <v>11798441.529999999</v>
+        <v>18500461.07</v>
       </c>
       <c r="G348" s="2">
         <v>348895.52</v>
       </c>
       <c r="H348" s="2">
-        <v>9375503.3900000006</v>
+        <v>14629547.470000001</v>
       </c>
       <c r="I348" s="2">
         <v>271878.39</v>
@@ -90588,11 +90598,11 @@
         <v>72</v>
       </c>
       <c r="F349" s="2">
-        <v>24959945.800000001</v>
+        <v>39508993.640000001</v>
       </c>
       <c r="G349"/>
       <c r="H349" s="2">
-        <v>19746182.57</v>
+        <v>31069593.640000001</v>
       </c>
       <c r="I349"/>
     </row>
@@ -90613,11 +90623,11 @@
         <v>73</v>
       </c>
       <c r="F350" s="2">
-        <v>43502093.960000001</v>
+        <v>76508520.25</v>
       </c>
       <c r="G350"/>
       <c r="H350" s="2">
-        <v>34040828.579999998</v>
+        <v>59820508.280000001</v>
       </c>
       <c r="I350"/>
     </row>
@@ -90638,22 +90648,22 @@
         <v>74</v>
       </c>
       <c r="F351" s="2">
-        <v>39019238.280000001</v>
+        <v>66398052.020000003</v>
       </c>
       <c r="G351" s="2">
-        <v>-270736.64000000001</v>
+        <v>2109104.3199999998</v>
       </c>
       <c r="H351" s="2">
-        <v>30807632.109999999</v>
+        <v>52477381.689999998</v>
       </c>
       <c r="I351" s="2">
-        <v>-212350.8</v>
+        <v>1652667.02</v>
       </c>
       <c r="J351" s="3">
-        <v>-113.946</v>
+        <v>535.72799999999995</v>
       </c>
       <c r="K351" s="3">
-        <v>2</v>
+        <v>18</v>
       </c>
     </row>
     <row r="352" spans="1:11" x14ac:dyDescent="0.25">
@@ -90673,13 +90683,23 @@
         <v>75</v>
       </c>
       <c r="F352" s="2">
-        <v>30834044.75</v>
-      </c>
-      <c r="G352"/>
+        <v>52444877.840000004</v>
+      </c>
+      <c r="G352">
+        <v>319999.2</v>
+      </c>
       <c r="H352" s="2">
-        <v>24094777.57</v>
-      </c>
-      <c r="I352"/>
+        <v>40981619.549999997</v>
+      </c>
+      <c r="I352">
+        <v>247933.26</v>
+      </c>
+      <c r="J352">
+        <v>1</v>
+      </c>
+      <c r="K352">
+        <v>1</v>
+      </c>
     </row>
     <row r="353" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A353" t="s">
@@ -90698,11 +90718,11 @@
         <v>76</v>
       </c>
       <c r="F353" s="2">
-        <v>35853797.229999997</v>
+        <v>59697635.5</v>
       </c>
       <c r="G353"/>
       <c r="H353" s="2">
-        <v>28147303.640000001</v>
+        <v>46771871.57</v>
       </c>
       <c r="I353"/>
     </row>
@@ -90723,11 +90743,11 @@
         <v>77</v>
       </c>
       <c r="F354" s="2">
-        <v>41159709.689999998</v>
+        <v>80092944.290000007</v>
       </c>
       <c r="G354"/>
       <c r="H354" s="2">
-        <v>32381413.329999998</v>
+        <v>62958212.920000002</v>
       </c>
       <c r="I354"/>
     </row>
@@ -90748,11 +90768,11 @@
         <v>78</v>
       </c>
       <c r="F355" s="2">
-        <v>42170899.229999997</v>
+        <v>65828887.609999999</v>
       </c>
       <c r="G355"/>
       <c r="H355" s="2">
-        <v>33082289.34</v>
+        <v>51651148.82</v>
       </c>
       <c r="I355"/>
     </row>
@@ -90773,11 +90793,11 @@
         <v>79</v>
       </c>
       <c r="F356" s="2">
-        <v>29832267.43</v>
+        <v>46893210.119999997</v>
       </c>
       <c r="G356"/>
       <c r="H356" s="2">
-        <v>23495781.199999999</v>
+        <v>36826435.590000004</v>
       </c>
       <c r="I356"/>
     </row>
@@ -90798,11 +90818,11 @@
         <v>81</v>
       </c>
       <c r="F357" s="2">
-        <v>55080034.060000002</v>
+        <v>84441532.870000005</v>
       </c>
       <c r="G357"/>
       <c r="H357" s="2">
-        <v>43934659.759999998</v>
+        <v>66949320.100000001</v>
       </c>
       <c r="I357"/>
     </row>
@@ -90823,11 +90843,11 @@
         <v>112</v>
       </c>
       <c r="F358" s="2">
-        <v>2225052.1</v>
+        <v>3980156.96</v>
       </c>
       <c r="G358"/>
       <c r="H358" s="2">
-        <v>1746479.75</v>
+        <v>3119580.84</v>
       </c>
       <c r="I358"/>
     </row>
@@ -90848,11 +90868,11 @@
         <v>83</v>
       </c>
       <c r="F359" s="2">
-        <v>21686687.32</v>
+        <v>37548564.670000002</v>
       </c>
       <c r="G359"/>
       <c r="H359" s="2">
-        <v>17207597.199999999</v>
+        <v>29575899.559999999</v>
       </c>
       <c r="I359"/>
     </row>
@@ -90873,13 +90893,23 @@
         <v>84</v>
       </c>
       <c r="F360" s="2">
-        <v>38512381.509999998</v>
-      </c>
-      <c r="G360"/>
+        <v>74492089.650000006</v>
+      </c>
+      <c r="G360">
+        <v>294054.40000000002</v>
+      </c>
       <c r="H360" s="2">
-        <v>30229136.350000001</v>
-      </c>
-      <c r="I360"/>
+        <v>58539586.670000002</v>
+      </c>
+      <c r="I360">
+        <v>226614.69</v>
+      </c>
+      <c r="J360">
+        <v>42.91</v>
+      </c>
+      <c r="K360">
+        <v>3</v>
+      </c>
     </row>
     <row r="361" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A361" t="s">
@@ -90898,11 +90928,11 @@
         <v>114</v>
       </c>
       <c r="F361" s="2">
-        <v>3244168.22</v>
+        <v>6719084.0199999996</v>
       </c>
       <c r="G361"/>
       <c r="H361" s="2">
-        <v>2548086.41</v>
+        <v>5214741.6399999997</v>
       </c>
       <c r="I361"/>
     </row>
@@ -90923,11 +90953,11 @@
         <v>85</v>
       </c>
       <c r="F362" s="2">
-        <v>23524673.309999999</v>
+        <v>40149230.219999999</v>
       </c>
       <c r="G362"/>
       <c r="H362" s="2">
-        <v>18553267.75</v>
+        <v>31578061.66</v>
       </c>
       <c r="I362"/>
     </row>
@@ -90948,13 +90978,13 @@
         <v>86</v>
       </c>
       <c r="F363" s="2">
-        <v>29154198.280000001</v>
+        <v>29232914.859999999</v>
       </c>
       <c r="G363" s="2">
         <v>1909997.38</v>
       </c>
       <c r="H363" s="2">
-        <v>23169010.52</v>
+        <v>23233772.579999998</v>
       </c>
       <c r="I363" s="2">
         <v>1479853.35</v>
@@ -90983,11 +91013,11 @@
         <v>87</v>
       </c>
       <c r="F364" s="2">
-        <v>21747983.059999999</v>
+        <v>38960602.670000002</v>
       </c>
       <c r="G364"/>
       <c r="H364" s="2">
-        <v>17118912.050000001</v>
+        <v>30635766.760000002</v>
       </c>
       <c r="I364"/>
     </row>
@@ -91008,11 +91038,11 @@
         <v>88</v>
       </c>
       <c r="F365" s="2">
-        <v>30771703.93</v>
+        <v>58078314.5</v>
       </c>
       <c r="G365"/>
       <c r="H365" s="2">
-        <v>24362370.09</v>
+        <v>45917569.329999998</v>
       </c>
       <c r="I365"/>
     </row>
@@ -91033,11 +91063,11 @@
         <v>89</v>
       </c>
       <c r="F366" s="2">
-        <v>31659307.289999999</v>
+        <v>51795539.829999998</v>
       </c>
       <c r="G366"/>
       <c r="H366" s="2">
-        <v>24922705.489999998</v>
+        <v>40765022.82</v>
       </c>
       <c r="I366"/>
     </row>
@@ -91058,11 +91088,11 @@
         <v>90</v>
       </c>
       <c r="F367" s="2">
-        <v>30806777.260000002</v>
+        <v>46932654.869999997</v>
       </c>
       <c r="G367"/>
       <c r="H367" s="2">
-        <v>24195790.579999998</v>
+        <v>36840850.310000002</v>
       </c>
       <c r="I367"/>
     </row>
@@ -91083,22 +91113,22 @@
         <v>91</v>
       </c>
       <c r="F368" s="2">
-        <v>167121641.97</v>
+        <v>286785298.66000003</v>
       </c>
       <c r="G368" s="2">
-        <v>4623692.3</v>
+        <v>6220219.3700000001</v>
       </c>
       <c r="H368" s="2">
-        <v>132927864.36</v>
+        <v>227448713.49000001</v>
       </c>
       <c r="I368" s="2">
-        <v>3595846.91</v>
+        <v>4837298.2699999996</v>
       </c>
       <c r="J368" s="3">
-        <v>1674.242</v>
+        <v>2159.8739999999998</v>
       </c>
       <c r="K368" s="3">
-        <v>54</v>
+        <v>65</v>
       </c>
     </row>
     <row r="369" spans="1:11" x14ac:dyDescent="0.25">
@@ -91118,13 +91148,13 @@
         <v>92</v>
       </c>
       <c r="F369" s="2">
-        <v>89086672.769999996</v>
+        <v>160993214.16999999</v>
       </c>
       <c r="G369" s="2">
         <v>4549077.72</v>
       </c>
       <c r="H369" s="2">
-        <v>69796426.730000004</v>
+        <v>125928765.91</v>
       </c>
       <c r="I369" s="2">
         <v>3495796.8</v>
@@ -91153,13 +91183,13 @@
         <v>93</v>
       </c>
       <c r="F370" s="2">
-        <v>82927643.439999998</v>
+        <v>167864342.31999999</v>
       </c>
       <c r="G370" s="2">
         <v>-62311.4</v>
       </c>
       <c r="H370" s="2">
-        <v>65118422.829999998</v>
+        <v>131707110.56</v>
       </c>
       <c r="I370" s="2">
         <v>-48278.47</v>
@@ -91188,22 +91218,22 @@
         <v>94</v>
       </c>
       <c r="F371" s="2">
-        <v>82409222.659999996</v>
+        <v>157918268.19999999</v>
       </c>
       <c r="G371" s="2">
-        <v>2314932.9900000002</v>
+        <v>3000653.86</v>
       </c>
       <c r="H371" s="2">
-        <v>64350092.729999997</v>
+        <v>123699521.52</v>
       </c>
       <c r="I371" s="2">
-        <v>1789502.88</v>
+        <v>2318835.4500000002</v>
       </c>
       <c r="J371" s="3">
-        <v>826.303</v>
+        <v>1032.462</v>
       </c>
       <c r="K371" s="3">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="372" spans="1:11" x14ac:dyDescent="0.25">
@@ -91223,11 +91253,11 @@
         <v>95</v>
       </c>
       <c r="F372" s="2">
-        <v>66582009.799999997</v>
+        <v>120776033.84</v>
       </c>
       <c r="G372"/>
       <c r="H372" s="2">
-        <v>52318261.649999999</v>
+        <v>94696480.640000001</v>
       </c>
       <c r="I372"/>
     </row>
@@ -91248,11 +91278,11 @@
         <v>96</v>
       </c>
       <c r="F373" s="2">
-        <v>89083836.430000007</v>
+        <v>205004352.74000001</v>
       </c>
       <c r="G373"/>
       <c r="H373" s="2">
-        <v>69683934.329999998</v>
+        <v>160089797.72999999</v>
       </c>
       <c r="I373"/>
     </row>
@@ -91273,11 +91303,11 @@
         <v>97</v>
       </c>
       <c r="F374" s="2">
-        <v>61991084.530000001</v>
+        <v>126763000.73</v>
       </c>
       <c r="G374"/>
       <c r="H374" s="2">
-        <v>48628458.939999998</v>
+        <v>99310339.120000005</v>
       </c>
       <c r="I374"/>
     </row>
@@ -91298,13 +91328,23 @@
         <v>98</v>
       </c>
       <c r="F375" s="2">
-        <v>108259870.11</v>
-      </c>
-      <c r="G375"/>
+        <v>186953093.02000001</v>
+      </c>
+      <c r="G375">
+        <v>4475833.83</v>
+      </c>
       <c r="H375" s="2">
-        <v>85499091.989999995</v>
-      </c>
-      <c r="I375"/>
+        <v>147308690.05000001</v>
+      </c>
+      <c r="I375">
+        <v>3457793.8</v>
+      </c>
+      <c r="J375">
+        <v>1326.921</v>
+      </c>
+      <c r="K375">
+        <v>36</v>
+      </c>
     </row>
     <row r="376" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A376" t="s">
@@ -91323,11 +91363,11 @@
         <v>99</v>
       </c>
       <c r="F376" s="2">
-        <v>75660184.219999999</v>
+        <v>137435044.59</v>
       </c>
       <c r="G376"/>
       <c r="H376" s="2">
-        <v>59621704.700000003</v>
+        <v>107956994.45</v>
       </c>
       <c r="I376"/>
     </row>
@@ -91348,13 +91388,13 @@
         <v>100</v>
       </c>
       <c r="F377" s="2">
-        <v>96443670.099999994</v>
+        <v>210955920.28999999</v>
       </c>
       <c r="G377" s="2">
         <v>1016637.9</v>
       </c>
       <c r="H377" s="2">
-        <v>75691404.650000006</v>
+        <v>164925455.52000001</v>
       </c>
       <c r="I377" s="2">
         <v>791361.49</v>
@@ -91383,13 +91423,23 @@
         <v>101</v>
       </c>
       <c r="F378" s="2">
-        <v>53152539.5</v>
-      </c>
-      <c r="G378"/>
+        <v>126811359.93000001</v>
+      </c>
+      <c r="G378">
+        <v>2262668.48</v>
+      </c>
       <c r="H378" s="2">
-        <v>41882872.640000001</v>
-      </c>
-      <c r="I378"/>
+        <v>99877139.640000001</v>
+      </c>
+      <c r="I378">
+        <v>1756773.73</v>
+      </c>
+      <c r="J378">
+        <v>754.11</v>
+      </c>
+      <c r="K378">
+        <v>12</v>
+      </c>
     </row>
     <row r="379" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A379" t="s">
@@ -91408,13 +91458,2749 @@
         <v>102</v>
       </c>
       <c r="F379" s="2">
-        <v>13226017.810000001</v>
+        <v>23687657.699999999</v>
       </c>
       <c r="G379"/>
       <c r="H379" s="2">
-        <v>10473150.32</v>
+        <v>18724006.18</v>
       </c>
       <c r="I379"/>
+    </row>
+    <row r="380" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A380" t="s">
+        <v>115</v>
+      </c>
+      <c r="B380" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C380" t="s">
+        <v>9</v>
+      </c>
+      <c r="D380">
+        <v>1002</v>
+      </c>
+      <c r="E380" t="s">
+        <v>10</v>
+      </c>
+      <c r="F380" s="4">
+        <v>67448514.370000005</v>
+      </c>
+      <c r="G380" s="4">
+        <v>2857806.22</v>
+      </c>
+      <c r="H380" s="4">
+        <v>52811215.170000002</v>
+      </c>
+      <c r="I380" s="4">
+        <v>2236997.11</v>
+      </c>
+      <c r="J380">
+        <v>918.48900000000003</v>
+      </c>
+      <c r="K380">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="381" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A381" t="s">
+        <v>115</v>
+      </c>
+      <c r="B381" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C381" t="s">
+        <v>9</v>
+      </c>
+      <c r="D381">
+        <v>1003</v>
+      </c>
+      <c r="E381" t="s">
+        <v>11</v>
+      </c>
+      <c r="F381" s="4">
+        <v>79190757.900000006</v>
+      </c>
+      <c r="G381" s="4">
+        <v>3174549.67</v>
+      </c>
+      <c r="H381" s="4">
+        <v>63156855.460000001</v>
+      </c>
+      <c r="I381" s="4">
+        <v>2490286.73</v>
+      </c>
+      <c r="J381">
+        <v>953.60900000000004</v>
+      </c>
+      <c r="K381">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="382" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A382" t="s">
+        <v>115</v>
+      </c>
+      <c r="B382" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C382" t="s">
+        <v>9</v>
+      </c>
+      <c r="D382">
+        <v>1004</v>
+      </c>
+      <c r="E382" t="s">
+        <v>12</v>
+      </c>
+      <c r="F382" s="4">
+        <v>104224072.16</v>
+      </c>
+      <c r="G382" s="4">
+        <v>4987541.5999999996</v>
+      </c>
+      <c r="H382" s="4">
+        <v>82288122.790000007</v>
+      </c>
+      <c r="I382" s="4">
+        <v>3949705.06</v>
+      </c>
+      <c r="J382">
+        <v>1333.298</v>
+      </c>
+      <c r="K382">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="383" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A383" t="s">
+        <v>115</v>
+      </c>
+      <c r="B383" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C383" t="s">
+        <v>9</v>
+      </c>
+      <c r="D383">
+        <v>1005</v>
+      </c>
+      <c r="E383" t="s">
+        <v>13</v>
+      </c>
+      <c r="F383" s="4">
+        <v>72624996.920000002</v>
+      </c>
+      <c r="H383" s="4">
+        <v>57769957.340000004</v>
+      </c>
+    </row>
+    <row r="384" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A384" t="s">
+        <v>115</v>
+      </c>
+      <c r="B384" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C384" t="s">
+        <v>9</v>
+      </c>
+      <c r="D384">
+        <v>1006</v>
+      </c>
+      <c r="E384" t="s">
+        <v>14</v>
+      </c>
+      <c r="F384" s="4">
+        <v>68493789.620000005</v>
+      </c>
+      <c r="G384" s="4">
+        <v>1916424.73</v>
+      </c>
+      <c r="H384" s="4">
+        <v>54521346.140000001</v>
+      </c>
+      <c r="I384" s="4">
+        <v>1499413.42</v>
+      </c>
+      <c r="J384">
+        <v>648.41700000000003</v>
+      </c>
+      <c r="K384">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="385" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A385" t="s">
+        <v>115</v>
+      </c>
+      <c r="B385" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C385" t="s">
+        <v>9</v>
+      </c>
+      <c r="D385">
+        <v>1007</v>
+      </c>
+      <c r="E385" t="s">
+        <v>15</v>
+      </c>
+      <c r="F385" s="4">
+        <v>88335522.900000006</v>
+      </c>
+      <c r="G385" s="4">
+        <v>523964.79</v>
+      </c>
+      <c r="H385" s="4">
+        <v>69765807.930000007</v>
+      </c>
+      <c r="I385" s="4">
+        <v>416806.3</v>
+      </c>
+      <c r="J385">
+        <v>156.77500000000001</v>
+      </c>
+      <c r="K385">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="386" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A386" t="s">
+        <v>115</v>
+      </c>
+      <c r="B386" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C386" t="s">
+        <v>9</v>
+      </c>
+      <c r="D386">
+        <v>1008</v>
+      </c>
+      <c r="E386" t="s">
+        <v>16</v>
+      </c>
+      <c r="F386" s="4">
+        <v>75976580.459999993</v>
+      </c>
+      <c r="G386" s="4">
+        <v>2310777.9700000002</v>
+      </c>
+      <c r="H386" s="4">
+        <v>59488191.560000002</v>
+      </c>
+      <c r="I386" s="4">
+        <v>1815231.77</v>
+      </c>
+      <c r="J386">
+        <v>483.05700000000002</v>
+      </c>
+      <c r="K386">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="387" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A387" t="s">
+        <v>115</v>
+      </c>
+      <c r="B387" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C387" t="s">
+        <v>9</v>
+      </c>
+      <c r="D387">
+        <v>1010</v>
+      </c>
+      <c r="E387" t="s">
+        <v>17</v>
+      </c>
+      <c r="F387" s="4">
+        <v>53028828.310000002</v>
+      </c>
+      <c r="H387" s="4">
+        <v>41781154.509999998</v>
+      </c>
+    </row>
+    <row r="388" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A388" t="s">
+        <v>115</v>
+      </c>
+      <c r="B388" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C388" t="s">
+        <v>9</v>
+      </c>
+      <c r="D388">
+        <v>1011</v>
+      </c>
+      <c r="E388" t="s">
+        <v>18</v>
+      </c>
+      <c r="F388" s="4">
+        <v>61759936.729999997</v>
+      </c>
+      <c r="G388" s="4">
+        <v>1334112.1000000001</v>
+      </c>
+      <c r="H388" s="4">
+        <v>48484704.939999998</v>
+      </c>
+      <c r="I388" s="4">
+        <v>1048114.14</v>
+      </c>
+      <c r="J388">
+        <v>294.25700000000001</v>
+      </c>
+      <c r="K388">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="389" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A389" t="s">
+        <v>115</v>
+      </c>
+      <c r="B389" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C389" t="s">
+        <v>9</v>
+      </c>
+      <c r="D389">
+        <v>1012</v>
+      </c>
+      <c r="E389" t="s">
+        <v>19</v>
+      </c>
+      <c r="F389" s="4">
+        <v>68780505.340000004</v>
+      </c>
+      <c r="G389" s="4">
+        <v>455724.46</v>
+      </c>
+      <c r="H389" s="4">
+        <v>53736947.640000001</v>
+      </c>
+      <c r="I389" s="4">
+        <v>355834.25</v>
+      </c>
+      <c r="J389">
+        <v>33.17</v>
+      </c>
+      <c r="K389">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="390" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A390" t="s">
+        <v>115</v>
+      </c>
+      <c r="B390" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C390" t="s">
+        <v>9</v>
+      </c>
+      <c r="D390">
+        <v>1013</v>
+      </c>
+      <c r="E390" t="s">
+        <v>20</v>
+      </c>
+      <c r="F390" s="4">
+        <v>49259715.109999999</v>
+      </c>
+      <c r="H390" s="4">
+        <v>38707955.020000003</v>
+      </c>
+    </row>
+    <row r="391" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A391" t="s">
+        <v>115</v>
+      </c>
+      <c r="B391" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C391" t="s">
+        <v>9</v>
+      </c>
+      <c r="D391">
+        <v>1014</v>
+      </c>
+      <c r="E391" t="s">
+        <v>21</v>
+      </c>
+      <c r="F391" s="4">
+        <v>47426307.490000002</v>
+      </c>
+      <c r="H391" s="4">
+        <v>37039971.07</v>
+      </c>
+    </row>
+    <row r="392" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A392" t="s">
+        <v>115</v>
+      </c>
+      <c r="B392" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C392" t="s">
+        <v>9</v>
+      </c>
+      <c r="D392">
+        <v>1015</v>
+      </c>
+      <c r="E392" t="s">
+        <v>22</v>
+      </c>
+      <c r="F392" s="4">
+        <v>59129754.270000003</v>
+      </c>
+      <c r="H392" s="4">
+        <v>46452717.200000003</v>
+      </c>
+    </row>
+    <row r="393" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A393" t="s">
+        <v>115</v>
+      </c>
+      <c r="B393" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C393" t="s">
+        <v>9</v>
+      </c>
+      <c r="D393">
+        <v>1016</v>
+      </c>
+      <c r="E393" t="s">
+        <v>23</v>
+      </c>
+      <c r="F393" s="4">
+        <v>63293643.789999999</v>
+      </c>
+      <c r="H393" s="4">
+        <v>49595684.100000001</v>
+      </c>
+    </row>
+    <row r="394" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A394" t="s">
+        <v>115</v>
+      </c>
+      <c r="B394" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C394" t="s">
+        <v>9</v>
+      </c>
+      <c r="D394">
+        <v>1017</v>
+      </c>
+      <c r="E394" t="s">
+        <v>24</v>
+      </c>
+      <c r="F394" s="4">
+        <v>52361107.979999997</v>
+      </c>
+      <c r="H394" s="4">
+        <v>40940129.289999999</v>
+      </c>
+    </row>
+    <row r="395" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A395" t="s">
+        <v>115</v>
+      </c>
+      <c r="B395" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C395" t="s">
+        <v>9</v>
+      </c>
+      <c r="D395">
+        <v>1018</v>
+      </c>
+      <c r="E395" t="s">
+        <v>25</v>
+      </c>
+      <c r="F395" s="4">
+        <v>51920440.079999998</v>
+      </c>
+      <c r="H395" s="4">
+        <v>40593190.920000002</v>
+      </c>
+    </row>
+    <row r="396" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A396" t="s">
+        <v>115</v>
+      </c>
+      <c r="B396" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C396" t="s">
+        <v>9</v>
+      </c>
+      <c r="D396">
+        <v>1020</v>
+      </c>
+      <c r="E396" t="s">
+        <v>26</v>
+      </c>
+      <c r="F396" s="4">
+        <v>73455731.040000007</v>
+      </c>
+      <c r="G396" s="4">
+        <v>4606344.3600000003</v>
+      </c>
+      <c r="H396" s="4">
+        <v>57986546.25</v>
+      </c>
+      <c r="I396" s="4">
+        <v>3589477.45</v>
+      </c>
+      <c r="J396">
+        <v>1306.2940000000001</v>
+      </c>
+      <c r="K396">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="397" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A397" t="s">
+        <v>115</v>
+      </c>
+      <c r="B397" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C397" t="s">
+        <v>9</v>
+      </c>
+      <c r="D397">
+        <v>1021</v>
+      </c>
+      <c r="E397" t="s">
+        <v>27</v>
+      </c>
+      <c r="F397" s="4">
+        <v>68191907.090000004</v>
+      </c>
+      <c r="H397" s="4">
+        <v>53306905.640000001</v>
+      </c>
+    </row>
+    <row r="398" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A398" t="s">
+        <v>115</v>
+      </c>
+      <c r="B398" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C398" t="s">
+        <v>9</v>
+      </c>
+      <c r="D398">
+        <v>1022</v>
+      </c>
+      <c r="E398" t="s">
+        <v>28</v>
+      </c>
+      <c r="F398" s="4">
+        <v>60538087.920000002</v>
+      </c>
+      <c r="G398" s="4">
+        <v>371175.74</v>
+      </c>
+      <c r="H398" s="4">
+        <v>48003233.390000001</v>
+      </c>
+      <c r="I398" s="4">
+        <v>289415.44</v>
+      </c>
+      <c r="J398">
+        <v>131.68700000000001</v>
+      </c>
+      <c r="K398">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="399" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A399" t="s">
+        <v>115</v>
+      </c>
+      <c r="B399" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C399" t="s">
+        <v>9</v>
+      </c>
+      <c r="D399">
+        <v>1023</v>
+      </c>
+      <c r="E399" t="s">
+        <v>29</v>
+      </c>
+      <c r="F399" s="4">
+        <v>45750857.530000001</v>
+      </c>
+      <c r="H399" s="4">
+        <v>35801412.840000004</v>
+      </c>
+    </row>
+    <row r="400" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A400" t="s">
+        <v>115</v>
+      </c>
+      <c r="B400" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C400" t="s">
+        <v>9</v>
+      </c>
+      <c r="D400">
+        <v>1024</v>
+      </c>
+      <c r="E400" t="s">
+        <v>30</v>
+      </c>
+      <c r="F400" s="4">
+        <v>65278697.590000004</v>
+      </c>
+      <c r="G400" s="4">
+        <v>3467853.76</v>
+      </c>
+      <c r="H400" s="4">
+        <v>51106512.990000002</v>
+      </c>
+      <c r="I400" s="4">
+        <v>2752727.74</v>
+      </c>
+      <c r="J400">
+        <v>1401.0989999999999</v>
+      </c>
+      <c r="K400">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="401" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A401" t="s">
+        <v>115</v>
+      </c>
+      <c r="B401" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C401" t="s">
+        <v>9</v>
+      </c>
+      <c r="D401">
+        <v>1026</v>
+      </c>
+      <c r="E401" t="s">
+        <v>31</v>
+      </c>
+      <c r="F401" s="4">
+        <v>46724190.710000001</v>
+      </c>
+      <c r="H401" s="4">
+        <v>36891138.619999997</v>
+      </c>
+    </row>
+    <row r="402" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A402" t="s">
+        <v>115</v>
+      </c>
+      <c r="B402" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C402" t="s">
+        <v>9</v>
+      </c>
+      <c r="D402">
+        <v>1027</v>
+      </c>
+      <c r="E402" t="s">
+        <v>32</v>
+      </c>
+      <c r="F402" s="4">
+        <v>17331507.079999998</v>
+      </c>
+      <c r="H402" s="4">
+        <v>13728883.91</v>
+      </c>
+    </row>
+    <row r="403" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A403" t="s">
+        <v>115</v>
+      </c>
+      <c r="B403" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C403" t="s">
+        <v>9</v>
+      </c>
+      <c r="D403">
+        <v>1028</v>
+      </c>
+      <c r="E403" t="s">
+        <v>33</v>
+      </c>
+      <c r="F403" s="4">
+        <v>41159435.259999998</v>
+      </c>
+      <c r="H403" s="4">
+        <v>32255111.190000001</v>
+      </c>
+    </row>
+    <row r="404" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A404" t="s">
+        <v>115</v>
+      </c>
+      <c r="B404" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C404" t="s">
+        <v>9</v>
+      </c>
+      <c r="D404">
+        <v>1029</v>
+      </c>
+      <c r="E404" t="s">
+        <v>34</v>
+      </c>
+      <c r="F404" s="4">
+        <v>34929469.159999996</v>
+      </c>
+      <c r="H404" s="4">
+        <v>27405082.010000002</v>
+      </c>
+    </row>
+    <row r="405" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A405" t="s">
+        <v>115</v>
+      </c>
+      <c r="B405" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C405" t="s">
+        <v>9</v>
+      </c>
+      <c r="D405">
+        <v>1030</v>
+      </c>
+      <c r="E405" t="s">
+        <v>35</v>
+      </c>
+      <c r="F405" s="4">
+        <v>15638475.49</v>
+      </c>
+      <c r="H405" s="4">
+        <v>12321787.029999999</v>
+      </c>
+    </row>
+    <row r="406" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A406" t="s">
+        <v>115</v>
+      </c>
+      <c r="B406" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C406" t="s">
+        <v>9</v>
+      </c>
+      <c r="D406">
+        <v>1031</v>
+      </c>
+      <c r="E406" t="s">
+        <v>36</v>
+      </c>
+      <c r="F406" s="4">
+        <v>72247304.689999998</v>
+      </c>
+      <c r="G406" s="4">
+        <v>1497303.52</v>
+      </c>
+      <c r="H406" s="4">
+        <v>56928508.450000003</v>
+      </c>
+      <c r="I406" s="4">
+        <v>1214833.24</v>
+      </c>
+      <c r="J406">
+        <v>439.35399999999998</v>
+      </c>
+      <c r="K406">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="407" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A407" t="s">
+        <v>115</v>
+      </c>
+      <c r="B407" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C407" t="s">
+        <v>9</v>
+      </c>
+      <c r="D407">
+        <v>1032</v>
+      </c>
+      <c r="E407" t="s">
+        <v>37</v>
+      </c>
+      <c r="F407" s="4">
+        <v>47667556.600000001</v>
+      </c>
+      <c r="H407" s="4">
+        <v>37394621.009999998</v>
+      </c>
+    </row>
+    <row r="408" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A408" t="s">
+        <v>115</v>
+      </c>
+      <c r="B408" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C408" t="s">
+        <v>9</v>
+      </c>
+      <c r="D408">
+        <v>1033</v>
+      </c>
+      <c r="E408" t="s">
+        <v>38</v>
+      </c>
+      <c r="F408" s="4">
+        <v>33330247.760000002</v>
+      </c>
+      <c r="G408" s="4">
+        <v>1688857.96</v>
+      </c>
+      <c r="H408" s="4">
+        <v>26378999.84</v>
+      </c>
+      <c r="I408" s="4">
+        <v>1309907.1399999999</v>
+      </c>
+      <c r="J408">
+        <v>18.065999999999999</v>
+      </c>
+      <c r="K408">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="409" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A409" t="s">
+        <v>115</v>
+      </c>
+      <c r="B409" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C409" t="s">
+        <v>9</v>
+      </c>
+      <c r="D409">
+        <v>1035</v>
+      </c>
+      <c r="E409" t="s">
+        <v>39</v>
+      </c>
+      <c r="F409" s="4">
+        <v>31003395.5</v>
+      </c>
+      <c r="H409" s="4">
+        <v>24332336.329999998</v>
+      </c>
+    </row>
+    <row r="410" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A410" t="s">
+        <v>115</v>
+      </c>
+      <c r="B410" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C410" t="s">
+        <v>9</v>
+      </c>
+      <c r="D410">
+        <v>1036</v>
+      </c>
+      <c r="E410" t="s">
+        <v>40</v>
+      </c>
+      <c r="F410" s="4">
+        <v>14949155.640000001</v>
+      </c>
+      <c r="H410" s="4">
+        <v>11715735.189999999</v>
+      </c>
+    </row>
+    <row r="411" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A411" t="s">
+        <v>115</v>
+      </c>
+      <c r="B411" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C411" t="s">
+        <v>9</v>
+      </c>
+      <c r="D411">
+        <v>1038</v>
+      </c>
+      <c r="E411" t="s">
+        <v>42</v>
+      </c>
+      <c r="F411" s="4">
+        <v>69445227.329999998</v>
+      </c>
+      <c r="G411" s="4">
+        <v>1959046.56</v>
+      </c>
+      <c r="H411" s="4">
+        <v>54352119.909999996</v>
+      </c>
+      <c r="I411" s="4">
+        <v>1551592.34</v>
+      </c>
+      <c r="J411">
+        <v>547.01</v>
+      </c>
+      <c r="K411">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="412" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A412" t="s">
+        <v>115</v>
+      </c>
+      <c r="B412" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C412" t="s">
+        <v>9</v>
+      </c>
+      <c r="D412">
+        <v>1039</v>
+      </c>
+      <c r="E412" t="s">
+        <v>43</v>
+      </c>
+      <c r="F412" s="4">
+        <v>58173783.700000003</v>
+      </c>
+      <c r="H412" s="4">
+        <v>45602357.539999999</v>
+      </c>
+    </row>
+    <row r="413" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A413" t="s">
+        <v>115</v>
+      </c>
+      <c r="B413" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C413" t="s">
+        <v>9</v>
+      </c>
+      <c r="D413">
+        <v>1042</v>
+      </c>
+      <c r="E413" t="s">
+        <v>44</v>
+      </c>
+      <c r="F413" s="4">
+        <v>42577555.740000002</v>
+      </c>
+      <c r="G413" s="4">
+        <v>2381555</v>
+      </c>
+      <c r="H413" s="4">
+        <v>33473280.289999999</v>
+      </c>
+      <c r="I413" s="4">
+        <v>1828474.43</v>
+      </c>
+      <c r="J413">
+        <v>186.131</v>
+      </c>
+      <c r="K413">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="414" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A414" t="s">
+        <v>115</v>
+      </c>
+      <c r="B414" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C414" t="s">
+        <v>9</v>
+      </c>
+      <c r="D414">
+        <v>1043</v>
+      </c>
+      <c r="E414" t="s">
+        <v>45</v>
+      </c>
+      <c r="F414" s="4">
+        <v>38352554.640000001</v>
+      </c>
+      <c r="H414" s="4">
+        <v>30047049.620000001</v>
+      </c>
+    </row>
+    <row r="415" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A415" t="s">
+        <v>115</v>
+      </c>
+      <c r="B415" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C415" t="s">
+        <v>9</v>
+      </c>
+      <c r="D415">
+        <v>1044</v>
+      </c>
+      <c r="E415" t="s">
+        <v>46</v>
+      </c>
+      <c r="F415" s="4">
+        <v>14212862.5</v>
+      </c>
+      <c r="H415" s="4">
+        <v>11146325.449999999</v>
+      </c>
+    </row>
+    <row r="416" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A416" t="s">
+        <v>115</v>
+      </c>
+      <c r="B416" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C416" t="s">
+        <v>9</v>
+      </c>
+      <c r="D416">
+        <v>1045</v>
+      </c>
+      <c r="E416" t="s">
+        <v>47</v>
+      </c>
+      <c r="F416" s="4">
+        <v>13572968.390000001</v>
+      </c>
+      <c r="H416" s="4">
+        <v>10698985.73</v>
+      </c>
+    </row>
+    <row r="417" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A417" t="s">
+        <v>115</v>
+      </c>
+      <c r="B417" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C417" t="s">
+        <v>9</v>
+      </c>
+      <c r="D417">
+        <v>1046</v>
+      </c>
+      <c r="E417" t="s">
+        <v>48</v>
+      </c>
+      <c r="F417" s="4">
+        <v>19906801.18</v>
+      </c>
+      <c r="H417" s="4">
+        <v>15607871.029999999</v>
+      </c>
+    </row>
+    <row r="418" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A418" t="s">
+        <v>115</v>
+      </c>
+      <c r="B418" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C418" t="s">
+        <v>9</v>
+      </c>
+      <c r="D418">
+        <v>1050</v>
+      </c>
+      <c r="E418" t="s">
+        <v>49</v>
+      </c>
+      <c r="F418" s="4">
+        <v>35914664.009999998</v>
+      </c>
+      <c r="H418" s="4">
+        <v>28125391.300000001</v>
+      </c>
+    </row>
+    <row r="419" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A419" t="s">
+        <v>115</v>
+      </c>
+      <c r="B419" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C419" t="s">
+        <v>9</v>
+      </c>
+      <c r="D419">
+        <v>1051</v>
+      </c>
+      <c r="E419" t="s">
+        <v>50</v>
+      </c>
+      <c r="F419" s="4">
+        <v>79750599.299999997</v>
+      </c>
+      <c r="G419" s="4">
+        <v>195462.9</v>
+      </c>
+      <c r="H419" s="4">
+        <v>63519372.219999999</v>
+      </c>
+      <c r="I419" s="4">
+        <v>149625.07</v>
+      </c>
+      <c r="J419">
+        <v>59.56</v>
+      </c>
+      <c r="K419">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="420" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A420" t="s">
+        <v>115</v>
+      </c>
+      <c r="B420" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C420" t="s">
+        <v>9</v>
+      </c>
+      <c r="D420">
+        <v>1052</v>
+      </c>
+      <c r="E420" t="s">
+        <v>51</v>
+      </c>
+      <c r="F420" s="4">
+        <v>35392656.880000003</v>
+      </c>
+      <c r="G420" s="4">
+        <v>105600.75</v>
+      </c>
+      <c r="H420" s="4">
+        <v>27854534.66</v>
+      </c>
+      <c r="I420" s="4">
+        <v>77944.84</v>
+      </c>
+      <c r="J420">
+        <v>17</v>
+      </c>
+      <c r="K420">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="421" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A421" t="s">
+        <v>115</v>
+      </c>
+      <c r="B421" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C421" t="s">
+        <v>9</v>
+      </c>
+      <c r="D421">
+        <v>1053</v>
+      </c>
+      <c r="E421" t="s">
+        <v>52</v>
+      </c>
+      <c r="F421" s="4">
+        <v>34443165.789999999</v>
+      </c>
+      <c r="H421" s="4">
+        <v>27029245</v>
+      </c>
+    </row>
+    <row r="422" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A422" t="s">
+        <v>115</v>
+      </c>
+      <c r="B422" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C422" t="s">
+        <v>9</v>
+      </c>
+      <c r="D422">
+        <v>1054</v>
+      </c>
+      <c r="E422" t="s">
+        <v>53</v>
+      </c>
+      <c r="F422" s="4">
+        <v>47403736.880000003</v>
+      </c>
+      <c r="G422" s="4">
+        <v>1635846.74</v>
+      </c>
+      <c r="H422" s="4">
+        <v>37095098.219999999</v>
+      </c>
+      <c r="I422" s="4">
+        <v>1300696.1499999999</v>
+      </c>
+      <c r="J422">
+        <v>419.62</v>
+      </c>
+      <c r="K422">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="423" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A423" t="s">
+        <v>115</v>
+      </c>
+      <c r="B423" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C423" t="s">
+        <v>9</v>
+      </c>
+      <c r="D423">
+        <v>1055</v>
+      </c>
+      <c r="E423" t="s">
+        <v>54</v>
+      </c>
+      <c r="F423" s="4">
+        <v>41169094.390000001</v>
+      </c>
+      <c r="G423" s="4">
+        <v>942482.11</v>
+      </c>
+      <c r="H423" s="4">
+        <v>32464285.640000001</v>
+      </c>
+      <c r="I423" s="4">
+        <v>739013.51</v>
+      </c>
+      <c r="J423">
+        <v>415.80599999999998</v>
+      </c>
+      <c r="K423">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="424" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A424" t="s">
+        <v>115</v>
+      </c>
+      <c r="B424" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C424" t="s">
+        <v>9</v>
+      </c>
+      <c r="D424">
+        <v>1056</v>
+      </c>
+      <c r="E424" t="s">
+        <v>55</v>
+      </c>
+      <c r="F424" s="4">
+        <v>41305335.460000001</v>
+      </c>
+      <c r="G424" s="4">
+        <v>44134.9</v>
+      </c>
+      <c r="H424" s="4">
+        <v>32440686.82</v>
+      </c>
+      <c r="I424" s="4">
+        <v>34195.43</v>
+      </c>
+      <c r="J424">
+        <v>24</v>
+      </c>
+      <c r="K424">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="425" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A425" t="s">
+        <v>115</v>
+      </c>
+      <c r="B425" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C425" t="s">
+        <v>9</v>
+      </c>
+      <c r="D425">
+        <v>1057</v>
+      </c>
+      <c r="E425" t="s">
+        <v>56</v>
+      </c>
+      <c r="F425" s="4">
+        <v>73237128.420000002</v>
+      </c>
+      <c r="G425" s="4">
+        <v>3828738.3</v>
+      </c>
+      <c r="H425" s="4">
+        <v>57615765.310000002</v>
+      </c>
+      <c r="I425" s="4">
+        <v>3059499.01</v>
+      </c>
+      <c r="J425">
+        <v>1167.039</v>
+      </c>
+      <c r="K425">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="426" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A426" t="s">
+        <v>115</v>
+      </c>
+      <c r="B426" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C426" t="s">
+        <v>9</v>
+      </c>
+      <c r="D426">
+        <v>1058</v>
+      </c>
+      <c r="E426" t="s">
+        <v>57</v>
+      </c>
+      <c r="F426" s="4">
+        <v>42966636.369999997</v>
+      </c>
+      <c r="G426" s="4">
+        <v>3679697.71</v>
+      </c>
+      <c r="H426" s="4">
+        <v>33394476.030000001</v>
+      </c>
+      <c r="I426" s="4">
+        <v>2851006.16</v>
+      </c>
+      <c r="J426">
+        <v>1160</v>
+      </c>
+      <c r="K426">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="427" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A427" t="s">
+        <v>115</v>
+      </c>
+      <c r="B427" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C427" t="s">
+        <v>9</v>
+      </c>
+      <c r="D427">
+        <v>1059</v>
+      </c>
+      <c r="E427" t="s">
+        <v>58</v>
+      </c>
+      <c r="F427" s="4">
+        <v>32265253.960000001</v>
+      </c>
+      <c r="H427" s="4">
+        <v>25243969.190000001</v>
+      </c>
+    </row>
+    <row r="428" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A428" t="s">
+        <v>115</v>
+      </c>
+      <c r="B428" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C428" t="s">
+        <v>9</v>
+      </c>
+      <c r="D428">
+        <v>1060</v>
+      </c>
+      <c r="E428" t="s">
+        <v>59</v>
+      </c>
+      <c r="F428" s="4">
+        <v>35547999.460000001</v>
+      </c>
+      <c r="H428" s="4">
+        <v>28326779.449999999</v>
+      </c>
+    </row>
+    <row r="429" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A429" t="s">
+        <v>115</v>
+      </c>
+      <c r="B429" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C429" t="s">
+        <v>9</v>
+      </c>
+      <c r="D429">
+        <v>1061</v>
+      </c>
+      <c r="E429" t="s">
+        <v>60</v>
+      </c>
+      <c r="F429" s="4">
+        <v>56910439.799999997</v>
+      </c>
+      <c r="G429" s="4">
+        <v>738526.35</v>
+      </c>
+      <c r="H429" s="4">
+        <v>44499893.460000001</v>
+      </c>
+      <c r="I429" s="4">
+        <v>569493.63</v>
+      </c>
+      <c r="J429">
+        <v>66</v>
+      </c>
+      <c r="K429">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="430" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A430" t="s">
+        <v>115</v>
+      </c>
+      <c r="B430" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C430" t="s">
+        <v>9</v>
+      </c>
+      <c r="D430">
+        <v>1066</v>
+      </c>
+      <c r="E430" t="s">
+        <v>111</v>
+      </c>
+      <c r="F430" s="4">
+        <v>2178929.0099999998</v>
+      </c>
+      <c r="H430" s="4">
+        <v>1696347.31</v>
+      </c>
+    </row>
+    <row r="431" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A431" t="s">
+        <v>115</v>
+      </c>
+      <c r="B431" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C431" t="s">
+        <v>9</v>
+      </c>
+      <c r="D431">
+        <v>1067</v>
+      </c>
+      <c r="E431" t="s">
+        <v>61</v>
+      </c>
+      <c r="F431" s="4">
+        <v>32151783.530000001</v>
+      </c>
+      <c r="G431" s="4">
+        <v>187200.61</v>
+      </c>
+      <c r="H431" s="4">
+        <v>25271770.600000001</v>
+      </c>
+      <c r="I431" s="4">
+        <v>145576.92000000001</v>
+      </c>
+      <c r="J431">
+        <v>60</v>
+      </c>
+      <c r="K431">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="432" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A432" t="s">
+        <v>115</v>
+      </c>
+      <c r="B432" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C432" t="s">
+        <v>9</v>
+      </c>
+      <c r="D432">
+        <v>1068</v>
+      </c>
+      <c r="E432" t="s">
+        <v>62</v>
+      </c>
+      <c r="F432" s="4">
+        <v>91753051.219999999</v>
+      </c>
+      <c r="H432" s="4">
+        <v>71959454.25</v>
+      </c>
+    </row>
+    <row r="433" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A433" t="s">
+        <v>115</v>
+      </c>
+      <c r="B433" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C433" t="s">
+        <v>9</v>
+      </c>
+      <c r="D433">
+        <v>1074</v>
+      </c>
+      <c r="E433" t="s">
+        <v>63</v>
+      </c>
+      <c r="F433" s="4">
+        <v>15393467.220000001</v>
+      </c>
+      <c r="G433" s="4">
+        <v>69000</v>
+      </c>
+      <c r="H433" s="4">
+        <v>12073634.369999999</v>
+      </c>
+      <c r="I433" s="4">
+        <v>49586.78</v>
+      </c>
+      <c r="J433">
+        <v>30</v>
+      </c>
+      <c r="K433">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="434" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A434" t="s">
+        <v>115</v>
+      </c>
+      <c r="B434" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C434" t="s">
+        <v>9</v>
+      </c>
+      <c r="D434">
+        <v>1075</v>
+      </c>
+      <c r="E434" t="s">
+        <v>64</v>
+      </c>
+      <c r="F434" s="4">
+        <v>47437845.329999998</v>
+      </c>
+      <c r="H434" s="4">
+        <v>37538153.850000001</v>
+      </c>
+    </row>
+    <row r="435" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A435" t="s">
+        <v>115</v>
+      </c>
+      <c r="B435" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C435" t="s">
+        <v>9</v>
+      </c>
+      <c r="D435">
+        <v>1076</v>
+      </c>
+      <c r="E435" t="s">
+        <v>65</v>
+      </c>
+      <c r="F435" s="4">
+        <v>43087893.049999997</v>
+      </c>
+      <c r="H435" s="4">
+        <v>33960383.57</v>
+      </c>
+    </row>
+    <row r="436" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A436" t="s">
+        <v>115</v>
+      </c>
+      <c r="B436" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C436" t="s">
+        <v>9</v>
+      </c>
+      <c r="D436">
+        <v>1077</v>
+      </c>
+      <c r="E436" t="s">
+        <v>66</v>
+      </c>
+      <c r="F436" s="4">
+        <v>52028513.020000003</v>
+      </c>
+      <c r="G436" s="4">
+        <v>635540.43000000005</v>
+      </c>
+      <c r="H436" s="4">
+        <v>40742834.200000003</v>
+      </c>
+      <c r="I436" s="4">
+        <v>496497.06</v>
+      </c>
+      <c r="J436">
+        <v>120.59099999999999</v>
+      </c>
+      <c r="K436">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="437" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A437" t="s">
+        <v>115</v>
+      </c>
+      <c r="B437" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C437" t="s">
+        <v>9</v>
+      </c>
+      <c r="D437">
+        <v>1078</v>
+      </c>
+      <c r="E437" t="s">
+        <v>67</v>
+      </c>
+      <c r="F437" s="4">
+        <v>43903735.109999999</v>
+      </c>
+      <c r="G437" s="4">
+        <v>784999.12</v>
+      </c>
+      <c r="H437" s="4">
+        <v>34242153.619999997</v>
+      </c>
+      <c r="I437" s="4">
+        <v>592716.26</v>
+      </c>
+      <c r="J437">
+        <v>1</v>
+      </c>
+      <c r="K437">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="438" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A438" t="s">
+        <v>115</v>
+      </c>
+      <c r="B438" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C438" t="s">
+        <v>9</v>
+      </c>
+      <c r="D438">
+        <v>1080</v>
+      </c>
+      <c r="E438" t="s">
+        <v>68</v>
+      </c>
+      <c r="F438" s="4">
+        <v>38886774.640000001</v>
+      </c>
+      <c r="G438" s="4">
+        <v>1623368.54</v>
+      </c>
+      <c r="H438" s="4">
+        <v>30316530.23</v>
+      </c>
+      <c r="I438" s="4">
+        <v>1292091.53</v>
+      </c>
+      <c r="J438">
+        <v>491.27</v>
+      </c>
+      <c r="K438">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="439" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A439" t="s">
+        <v>115</v>
+      </c>
+      <c r="B439" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C439" t="s">
+        <v>9</v>
+      </c>
+      <c r="D439">
+        <v>1081</v>
+      </c>
+      <c r="E439" t="s">
+        <v>69</v>
+      </c>
+      <c r="F439" s="4">
+        <v>34380699.439999998</v>
+      </c>
+      <c r="H439" s="4">
+        <v>27176756.629999999</v>
+      </c>
+    </row>
+    <row r="440" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A440" t="s">
+        <v>115</v>
+      </c>
+      <c r="B440" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C440" t="s">
+        <v>9</v>
+      </c>
+      <c r="D440">
+        <v>1082</v>
+      </c>
+      <c r="E440" t="s">
+        <v>70</v>
+      </c>
+      <c r="F440" s="4">
+        <v>15100898.42</v>
+      </c>
+      <c r="H440" s="4">
+        <v>11947943.4</v>
+      </c>
+    </row>
+    <row r="441" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A441" t="s">
+        <v>115</v>
+      </c>
+      <c r="B441" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C441" t="s">
+        <v>9</v>
+      </c>
+      <c r="D441">
+        <v>1084</v>
+      </c>
+      <c r="E441" t="s">
+        <v>71</v>
+      </c>
+      <c r="F441" s="4">
+        <v>12358456.99</v>
+      </c>
+      <c r="H441" s="4">
+        <v>9700556.8800000008</v>
+      </c>
+    </row>
+    <row r="442" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A442" t="s">
+        <v>115</v>
+      </c>
+      <c r="B442" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C442" t="s">
+        <v>9</v>
+      </c>
+      <c r="D442">
+        <v>1085</v>
+      </c>
+      <c r="E442" t="s">
+        <v>72</v>
+      </c>
+      <c r="F442" s="4">
+        <v>19827623.5</v>
+      </c>
+      <c r="H442" s="4">
+        <v>15491710.66</v>
+      </c>
+    </row>
+    <row r="443" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A443" t="s">
+        <v>115</v>
+      </c>
+      <c r="B443" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C443" t="s">
+        <v>9</v>
+      </c>
+      <c r="D443">
+        <v>1086</v>
+      </c>
+      <c r="E443" t="s">
+        <v>73</v>
+      </c>
+      <c r="F443" s="4">
+        <v>36928255.649999999</v>
+      </c>
+      <c r="H443" s="4">
+        <v>28818448.350000001</v>
+      </c>
+    </row>
+    <row r="444" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A444" t="s">
+        <v>115</v>
+      </c>
+      <c r="B444" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C444" t="s">
+        <v>9</v>
+      </c>
+      <c r="D444">
+        <v>1087</v>
+      </c>
+      <c r="E444" t="s">
+        <v>74</v>
+      </c>
+      <c r="F444" s="4">
+        <v>71187131.269999996</v>
+      </c>
+      <c r="G444" s="4">
+        <v>4748492.82</v>
+      </c>
+      <c r="H444" s="4">
+        <v>55977482.960000001</v>
+      </c>
+      <c r="I444" s="4">
+        <v>3714698.86</v>
+      </c>
+      <c r="J444">
+        <v>1407.2850000000001</v>
+      </c>
+      <c r="K444">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="445" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A445" t="s">
+        <v>115</v>
+      </c>
+      <c r="B445" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C445" t="s">
+        <v>9</v>
+      </c>
+      <c r="D445">
+        <v>1088</v>
+      </c>
+      <c r="E445" t="s">
+        <v>75</v>
+      </c>
+      <c r="F445" s="4">
+        <v>37897777.57</v>
+      </c>
+      <c r="H445" s="4">
+        <v>30561161.550000001</v>
+      </c>
+    </row>
+    <row r="446" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A446" t="s">
+        <v>115</v>
+      </c>
+      <c r="B446" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C446" t="s">
+        <v>9</v>
+      </c>
+      <c r="D446">
+        <v>1092</v>
+      </c>
+      <c r="E446" t="s">
+        <v>76</v>
+      </c>
+      <c r="F446" s="4">
+        <v>43702376.329999998</v>
+      </c>
+      <c r="G446" s="4">
+        <v>1199999.25</v>
+      </c>
+      <c r="H446" s="4">
+        <v>34076997.710000001</v>
+      </c>
+      <c r="I446" s="4">
+        <v>929751.51</v>
+      </c>
+      <c r="J446">
+        <v>1</v>
+      </c>
+      <c r="K446">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="447" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A447" t="s">
+        <v>115</v>
+      </c>
+      <c r="B447" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C447" t="s">
+        <v>9</v>
+      </c>
+      <c r="D447">
+        <v>1093</v>
+      </c>
+      <c r="E447" t="s">
+        <v>77</v>
+      </c>
+      <c r="F447" s="4">
+        <v>59219789.719999999</v>
+      </c>
+      <c r="H447" s="4">
+        <v>46620339.280000001</v>
+      </c>
+    </row>
+    <row r="448" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A448" t="s">
+        <v>115</v>
+      </c>
+      <c r="B448" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C448" t="s">
+        <v>9</v>
+      </c>
+      <c r="D448">
+        <v>1096</v>
+      </c>
+      <c r="E448" t="s">
+        <v>78</v>
+      </c>
+      <c r="F448" s="4">
+        <v>44977363.57</v>
+      </c>
+      <c r="H448" s="4">
+        <v>35362712.409999996</v>
+      </c>
+    </row>
+    <row r="449" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A449" t="s">
+        <v>115</v>
+      </c>
+      <c r="B449" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C449" t="s">
+        <v>9</v>
+      </c>
+      <c r="D449">
+        <v>1097</v>
+      </c>
+      <c r="E449" t="s">
+        <v>79</v>
+      </c>
+      <c r="F449" s="4">
+        <v>33183236.73</v>
+      </c>
+      <c r="H449" s="4">
+        <v>26173017.879999999</v>
+      </c>
+    </row>
+    <row r="450" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A450" t="s">
+        <v>115</v>
+      </c>
+      <c r="B450" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C450" t="s">
+        <v>9</v>
+      </c>
+      <c r="D450">
+        <v>1098</v>
+      </c>
+      <c r="E450" t="s">
+        <v>80</v>
+      </c>
+      <c r="F450" s="4">
+        <v>22248946.969999999</v>
+      </c>
+      <c r="H450" s="4">
+        <v>17362240.5</v>
+      </c>
+    </row>
+    <row r="451" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A451" t="s">
+        <v>115</v>
+      </c>
+      <c r="B451" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C451" t="s">
+        <v>9</v>
+      </c>
+      <c r="D451">
+        <v>1099</v>
+      </c>
+      <c r="E451" t="s">
+        <v>81</v>
+      </c>
+      <c r="F451" s="4">
+        <v>34732898.229999997</v>
+      </c>
+      <c r="G451" s="4">
+        <v>204999</v>
+      </c>
+      <c r="H451" s="4">
+        <v>27832238.059999999</v>
+      </c>
+      <c r="I451" s="4">
+        <v>158831.87</v>
+      </c>
+      <c r="J451">
+        <v>1</v>
+      </c>
+      <c r="K451">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="452" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A452" t="s">
+        <v>115</v>
+      </c>
+      <c r="B452" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C452" t="s">
+        <v>9</v>
+      </c>
+      <c r="D452">
+        <v>1100</v>
+      </c>
+      <c r="E452" t="s">
+        <v>82</v>
+      </c>
+      <c r="F452" s="4">
+        <v>37049536.359999999</v>
+      </c>
+      <c r="H452" s="4">
+        <v>29124376.210000001</v>
+      </c>
+    </row>
+    <row r="453" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A453" t="s">
+        <v>115</v>
+      </c>
+      <c r="B453" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C453" t="s">
+        <v>9</v>
+      </c>
+      <c r="D453">
+        <v>1102</v>
+      </c>
+      <c r="E453" t="s">
+        <v>112</v>
+      </c>
+      <c r="F453" s="4">
+        <v>2484491.86</v>
+      </c>
+      <c r="H453" s="4">
+        <v>1939097.03</v>
+      </c>
+    </row>
+    <row r="454" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A454" t="s">
+        <v>115</v>
+      </c>
+      <c r="B454" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C454" t="s">
+        <v>9</v>
+      </c>
+      <c r="D454">
+        <v>1103</v>
+      </c>
+      <c r="E454" t="s">
+        <v>113</v>
+      </c>
+      <c r="F454" s="4">
+        <v>3431028.75</v>
+      </c>
+      <c r="H454" s="4">
+        <v>2674351.2000000002</v>
+      </c>
+    </row>
+    <row r="455" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A455" t="s">
+        <v>115</v>
+      </c>
+      <c r="B455" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C455" t="s">
+        <v>9</v>
+      </c>
+      <c r="D455">
+        <v>1106</v>
+      </c>
+      <c r="E455" t="s">
+        <v>83</v>
+      </c>
+      <c r="F455" s="4">
+        <v>18822712.5</v>
+      </c>
+      <c r="H455" s="4">
+        <v>14778846.23</v>
+      </c>
+    </row>
+    <row r="456" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A456" t="s">
+        <v>115</v>
+      </c>
+      <c r="B456" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C456" t="s">
+        <v>9</v>
+      </c>
+      <c r="D456">
+        <v>1108</v>
+      </c>
+      <c r="E456" t="s">
+        <v>84</v>
+      </c>
+      <c r="F456" s="4">
+        <v>44955894.310000002</v>
+      </c>
+      <c r="G456" s="4">
+        <v>192953</v>
+      </c>
+      <c r="H456" s="4">
+        <v>35389225.32</v>
+      </c>
+      <c r="I456" s="4">
+        <v>155989.37</v>
+      </c>
+      <c r="J456">
+        <v>61.701999999999998</v>
+      </c>
+      <c r="K456">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="457" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A457" t="s">
+        <v>115</v>
+      </c>
+      <c r="B457" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C457" t="s">
+        <v>9</v>
+      </c>
+      <c r="D457">
+        <v>1109</v>
+      </c>
+      <c r="E457" t="s">
+        <v>114</v>
+      </c>
+      <c r="F457" s="4">
+        <v>2920548.05</v>
+      </c>
+      <c r="H457" s="4">
+        <v>2281325.66</v>
+      </c>
+    </row>
+    <row r="458" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A458" t="s">
+        <v>115</v>
+      </c>
+      <c r="B458" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C458" t="s">
+        <v>9</v>
+      </c>
+      <c r="D458">
+        <v>1110</v>
+      </c>
+      <c r="E458" t="s">
+        <v>85</v>
+      </c>
+      <c r="F458" s="4">
+        <v>21798931.739999998</v>
+      </c>
+      <c r="H458" s="4">
+        <v>17108826.670000002</v>
+      </c>
+    </row>
+    <row r="459" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A459" t="s">
+        <v>115</v>
+      </c>
+      <c r="B459" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C459" t="s">
+        <v>9</v>
+      </c>
+      <c r="D459">
+        <v>1111</v>
+      </c>
+      <c r="E459" t="s">
+        <v>86</v>
+      </c>
+      <c r="F459" s="4">
+        <v>23865124.760000002</v>
+      </c>
+      <c r="H459" s="4">
+        <v>18769817.079999998</v>
+      </c>
+    </row>
+    <row r="460" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A460" t="s">
+        <v>115</v>
+      </c>
+      <c r="B460" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C460" t="s">
+        <v>9</v>
+      </c>
+      <c r="D460">
+        <v>1114</v>
+      </c>
+      <c r="E460" t="s">
+        <v>87</v>
+      </c>
+      <c r="F460" s="4">
+        <v>23682976.84</v>
+      </c>
+      <c r="H460" s="4">
+        <v>18538557.07</v>
+      </c>
+    </row>
+    <row r="461" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A461" t="s">
+        <v>115</v>
+      </c>
+      <c r="B461" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C461" t="s">
+        <v>9</v>
+      </c>
+      <c r="D461">
+        <v>1115</v>
+      </c>
+      <c r="E461" t="s">
+        <v>88</v>
+      </c>
+      <c r="F461" s="4">
+        <v>39932253.32</v>
+      </c>
+      <c r="G461" s="4">
+        <v>775691.04</v>
+      </c>
+      <c r="H461" s="4">
+        <v>31488483.34</v>
+      </c>
+      <c r="I461" s="4">
+        <v>612857.23</v>
+      </c>
+      <c r="J461">
+        <v>266.73</v>
+      </c>
+      <c r="K461">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="462" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A462" t="s">
+        <v>115</v>
+      </c>
+      <c r="B462" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C462" t="s">
+        <v>9</v>
+      </c>
+      <c r="D462">
+        <v>1116</v>
+      </c>
+      <c r="E462" t="s">
+        <v>89</v>
+      </c>
+      <c r="F462" s="4">
+        <v>31502965.699999999</v>
+      </c>
+      <c r="H462" s="4">
+        <v>24727677.82</v>
+      </c>
+    </row>
+    <row r="463" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A463" t="s">
+        <v>115</v>
+      </c>
+      <c r="B463" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C463" t="s">
+        <v>9</v>
+      </c>
+      <c r="D463">
+        <v>1119</v>
+      </c>
+      <c r="E463" t="s">
+        <v>90</v>
+      </c>
+      <c r="F463" s="4">
+        <v>20544057.140000001</v>
+      </c>
+      <c r="H463" s="4">
+        <v>16085366.130000001</v>
+      </c>
+    </row>
+    <row r="464" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A464" t="s">
+        <v>115</v>
+      </c>
+      <c r="B464" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C464" t="s">
+        <v>9</v>
+      </c>
+      <c r="D464">
+        <v>2997</v>
+      </c>
+      <c r="E464" t="s">
+        <v>91</v>
+      </c>
+      <c r="F464" s="4">
+        <v>241889697.61000001</v>
+      </c>
+      <c r="G464" s="4">
+        <v>22493405.199999999</v>
+      </c>
+      <c r="H464" s="4">
+        <v>192761532.61000001</v>
+      </c>
+      <c r="I464" s="4">
+        <v>17495564.300000001</v>
+      </c>
+      <c r="J464">
+        <v>6577.8130000000001</v>
+      </c>
+      <c r="K464">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="465" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A465" t="s">
+        <v>115</v>
+      </c>
+      <c r="B465" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C465" t="s">
+        <v>9</v>
+      </c>
+      <c r="D465">
+        <v>2998</v>
+      </c>
+      <c r="E465" t="s">
+        <v>92</v>
+      </c>
+      <c r="F465" s="4">
+        <v>100340877.77</v>
+      </c>
+      <c r="G465" s="4">
+        <v>12071621.35</v>
+      </c>
+      <c r="H465" s="4">
+        <v>78371793.510000005</v>
+      </c>
+      <c r="I465" s="4">
+        <v>9381145.9900000002</v>
+      </c>
+      <c r="J465">
+        <v>4094</v>
+      </c>
+      <c r="K465">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="466" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A466" t="s">
+        <v>115</v>
+      </c>
+      <c r="B466" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C466" t="s">
+        <v>9</v>
+      </c>
+      <c r="D466">
+        <v>2999</v>
+      </c>
+      <c r="E466" t="s">
+        <v>93</v>
+      </c>
+      <c r="F466" s="4">
+        <v>109477974.09999999</v>
+      </c>
+      <c r="G466" s="4">
+        <v>10933837.640000001</v>
+      </c>
+      <c r="H466" s="4">
+        <v>85602512.510000005</v>
+      </c>
+      <c r="I466" s="4">
+        <v>8494776.7400000002</v>
+      </c>
+      <c r="J466">
+        <v>3419.3229999999999</v>
+      </c>
+      <c r="K466">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="467" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A467" t="s">
+        <v>115</v>
+      </c>
+      <c r="B467" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C467" t="s">
+        <v>9</v>
+      </c>
+      <c r="D467">
+        <v>3601</v>
+      </c>
+      <c r="E467" t="s">
+        <v>94</v>
+      </c>
+      <c r="F467" s="4">
+        <v>136002132.87</v>
+      </c>
+      <c r="G467" s="4">
+        <v>11599242.380000001</v>
+      </c>
+      <c r="H467" s="4">
+        <v>106478260.76000001</v>
+      </c>
+      <c r="I467" s="4">
+        <v>9013348.0800000001</v>
+      </c>
+      <c r="J467">
+        <v>3823.4110000000001</v>
+      </c>
+      <c r="K467">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="468" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A468" t="s">
+        <v>115</v>
+      </c>
+      <c r="B468" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C468" t="s">
+        <v>9</v>
+      </c>
+      <c r="D468">
+        <v>3602</v>
+      </c>
+      <c r="E468" t="s">
+        <v>95</v>
+      </c>
+      <c r="F468" s="4">
+        <v>120412076.77</v>
+      </c>
+      <c r="G468" s="4">
+        <v>7361323.9900000002</v>
+      </c>
+      <c r="H468" s="4">
+        <v>94344890.980000004</v>
+      </c>
+      <c r="I468" s="4">
+        <v>5702035.4800000004</v>
+      </c>
+      <c r="J468">
+        <v>1803.644</v>
+      </c>
+      <c r="K468">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="469" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A469" t="s">
+        <v>115</v>
+      </c>
+      <c r="B469" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C469" t="s">
+        <v>9</v>
+      </c>
+      <c r="D469">
+        <v>3603</v>
+      </c>
+      <c r="E469" t="s">
+        <v>96</v>
+      </c>
+      <c r="F469" s="4">
+        <v>115237654.79000001</v>
+      </c>
+      <c r="G469" s="4">
+        <v>4938615.1399999997</v>
+      </c>
+      <c r="H469" s="4">
+        <v>90254124.469999999</v>
+      </c>
+      <c r="I469" s="4">
+        <v>3826863.1</v>
+      </c>
+      <c r="J469">
+        <v>1528.4469999999999</v>
+      </c>
+      <c r="K469">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="470" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A470" t="s">
+        <v>115</v>
+      </c>
+      <c r="B470" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C470" t="s">
+        <v>9</v>
+      </c>
+      <c r="D470">
+        <v>3604</v>
+      </c>
+      <c r="E470" t="s">
+        <v>97</v>
+      </c>
+      <c r="F470" s="4">
+        <v>69573379.040000007</v>
+      </c>
+      <c r="G470" s="4">
+        <v>8806264.4800000004</v>
+      </c>
+      <c r="H470" s="4">
+        <v>54623082.850000001</v>
+      </c>
+      <c r="I470" s="4">
+        <v>6793807.0599999996</v>
+      </c>
+      <c r="J470">
+        <v>1784.588</v>
+      </c>
+      <c r="K470">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="471" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A471" t="s">
+        <v>115</v>
+      </c>
+      <c r="B471" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C471" t="s">
+        <v>9</v>
+      </c>
+      <c r="D471">
+        <v>3605</v>
+      </c>
+      <c r="E471" t="s">
+        <v>98</v>
+      </c>
+      <c r="F471" s="4">
+        <v>173556013.97999999</v>
+      </c>
+      <c r="G471" s="4">
+        <v>15394914.59</v>
+      </c>
+      <c r="H471" s="4">
+        <v>136990140.88999999</v>
+      </c>
+      <c r="I471" s="4">
+        <v>11949824.25</v>
+      </c>
+      <c r="J471">
+        <v>4216.2920000000004</v>
+      </c>
+      <c r="K471">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="472" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A472" t="s">
+        <v>115</v>
+      </c>
+      <c r="B472" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C472" t="s">
+        <v>9</v>
+      </c>
+      <c r="D472">
+        <v>3606</v>
+      </c>
+      <c r="E472" t="s">
+        <v>99</v>
+      </c>
+      <c r="F472" s="4">
+        <v>86054597.590000004</v>
+      </c>
+      <c r="H472" s="4">
+        <v>67725247.239999995</v>
+      </c>
+    </row>
+    <row r="473" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A473" t="s">
+        <v>115</v>
+      </c>
+      <c r="B473" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C473" t="s">
+        <v>9</v>
+      </c>
+      <c r="D473">
+        <v>3608</v>
+      </c>
+      <c r="E473" t="s">
+        <v>100</v>
+      </c>
+      <c r="F473" s="4">
+        <v>125246388.63</v>
+      </c>
+      <c r="G473" s="4">
+        <v>4237502.97</v>
+      </c>
+      <c r="H473" s="4">
+        <v>97578594.370000005</v>
+      </c>
+      <c r="I473" s="4">
+        <v>3333050.55</v>
+      </c>
+      <c r="J473">
+        <v>1175.903</v>
+      </c>
+      <c r="K473">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="474" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A474" t="s">
+        <v>115</v>
+      </c>
+      <c r="B474" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C474" t="s">
+        <v>9</v>
+      </c>
+      <c r="D474">
+        <v>3613</v>
+      </c>
+      <c r="E474" t="s">
+        <v>101</v>
+      </c>
+      <c r="F474" s="4">
+        <v>121393592.06999999</v>
+      </c>
+      <c r="G474" s="4">
+        <v>9000407.8800000008</v>
+      </c>
+      <c r="H474" s="4">
+        <v>95800738.920000002</v>
+      </c>
+      <c r="I474" s="4">
+        <v>7029934.8200000003</v>
+      </c>
+      <c r="J474">
+        <v>2833.3890000000001</v>
+      </c>
+      <c r="K474">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="475" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A475" t="s">
+        <v>115</v>
+      </c>
+      <c r="B475" s="5">
+        <v>46300</v>
+      </c>
+      <c r="C475" t="s">
+        <v>9</v>
+      </c>
+      <c r="D475">
+        <v>4001</v>
+      </c>
+      <c r="E475" t="s">
+        <v>102</v>
+      </c>
+      <c r="F475" s="4">
+        <v>20166128.890000001</v>
+      </c>
+      <c r="G475" s="4">
+        <v>31242.75</v>
+      </c>
+      <c r="H475" s="4">
+        <v>15877252.41</v>
+      </c>
+      <c r="I475" s="4">
+        <v>26236.26</v>
+      </c>
+      <c r="J475">
+        <v>13</v>
+      </c>
+      <c r="K475">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K1" xr:uid="{FE92DB44-9108-48C0-9E4D-CDD7D4A1EECC}"/>

</xml_diff>